<commit_message>
mantine 7 upgrade 22feb
</commit_message>
<xml_diff>
--- a/timesheet/T26TimeSheet_chanaa_FEB2024.xlsx
+++ b/timesheet/T26TimeSheet_chanaa_FEB2024.xlsx
@@ -52,7 +52,7 @@
     <t>Post Unit</t>
   </si>
   <si>
-    <t>unit1</t>
+    <t>unit11</t>
   </si>
   <si>
     <t>Timesheet Start Date</t>
@@ -88,7 +88,7 @@
     <t>Email</t>
   </si>
   <si>
-    <t>a@a.com</t>
+    <t>x@a.com</t>
   </si>
   <si>
     <t>Commitment Ref.(if applicable)</t>

</xml_diff>

<commit_message>
Fix timesheet, help user to go to init calendar when the calendar DB is not initialized.
</commit_message>
<xml_diff>
--- a/timesheet/T26TimeSheet_chanaa_FEB2024.xlsx
+++ b/timesheet/T26TimeSheet_chanaa_FEB2024.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="66">
   <si>
     <t>Contract Ref.: GCIO 5/2 (T26)</t>
   </si>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="B25" s="52"/>
       <c r="C25" s="53">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="D25" s="53"/>
       <c r="E25" s="53">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="I25" s="53"/>
       <c r="J25" s="53">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K25" s="53"/>
       <c r="L25" s="53">
@@ -2136,7 +2136,7 @@
       </c>
       <c r="B35" s="52"/>
       <c r="C35" s="53">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D35" s="53"/>
       <c r="E35" s="53">
@@ -2153,7 +2153,7 @@
       </c>
       <c r="K35" s="53"/>
       <c r="L35" s="53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M35" s="53"/>
       <c r="N35" s="53">
@@ -2198,7 +2198,7 @@
       </c>
       <c r="B37" s="52"/>
       <c r="C37" s="53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D37" s="53"/>
       <c r="E37" s="53">
@@ -2215,7 +2215,7 @@
       </c>
       <c r="K37" s="53"/>
       <c r="L37" s="53">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M37" s="53"/>
       <c r="N37" s="53">
@@ -2353,7 +2353,7 @@
       </c>
       <c r="B42" s="52"/>
       <c r="C42" s="53">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D42" s="53"/>
       <c r="E42" s="53">
@@ -2370,7 +2370,7 @@
       </c>
       <c r="K42" s="53"/>
       <c r="L42" s="53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M42" s="53"/>
       <c r="N42" s="53">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="B44" s="52"/>
       <c r="C44" s="53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D44" s="53"/>
       <c r="E44" s="53">
@@ -2432,7 +2432,7 @@
       </c>
       <c r="K44" s="53"/>
       <c r="L44" s="53">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M44" s="53"/>
       <c r="N44" s="53">
@@ -2534,33 +2534,33 @@
       <c r="O47" s="53"/>
     </row>
     <row r="48" ht="12" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A48" s="52" t="s">
-        <v>42</v>
+      <c r="A48" s="52">
+        <v>29</v>
       </c>
       <c r="B48" s="52"/>
-      <c r="C48" s="53" t="s">
-        <v>42</v>
+      <c r="C48" s="53">
+        <v>1</v>
       </c>
       <c r="D48" s="53"/>
-      <c r="E48" s="53" t="s">
-        <v>42</v>
+      <c r="E48" s="53">
+        <v>0</v>
       </c>
       <c r="F48" s="53"/>
       <c r="G48" s="53"/>
-      <c r="H48" s="53" t="s">
-        <v>42</v>
+      <c r="H48" s="53">
+        <v>0</v>
       </c>
       <c r="I48" s="53"/>
-      <c r="J48" s="53" t="s">
-        <v>42</v>
+      <c r="J48" s="53">
+        <v>0</v>
       </c>
       <c r="K48" s="53"/>
-      <c r="L48" s="53" t="s">
-        <v>42</v>
+      <c r="L48" s="53">
+        <v>0</v>
       </c>
       <c r="M48" s="53"/>
-      <c r="N48" s="53" t="s">
-        <v>42</v>
+      <c r="N48" s="53">
+        <v>0</v>
       </c>
       <c r="O48" s="53"/>
     </row>
@@ -2632,7 +2632,7 @@
       </c>
       <c r="B51" s="56"/>
       <c r="C51" s="53">
-        <v>15</v>
+        <v>15.5</v>
       </c>
       <c r="D51" s="52"/>
       <c r="E51" s="53">

</xml_diff>